<commit_message>
Refactor CPI data acquisition and transformation
- Updated acquire.py to fetch national annual CPI data instead of state-level monthly data.
- Changed configuration in config.py to reflect the new national CPI CSV source.
- Modified transform.py to build a national annual CPI table, removing state-specific logic.
- Adjusted visualisation.py for consistent color mapping and legend handling.
</commit_message>
<xml_diff>
--- a/data/clean/dashboard_data.xlsx
+++ b/data/clean/dashboard_data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="sdi_scores" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="combined_state" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="health_state" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="cpi_state" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="cpi_national" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1638,7 +1638,9 @@
         <v>45.7</v>
       </c>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="n">
+        <v>23.3563585414548</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1669,7 +1671,9 @@
       <c r="H3" t="n">
         <v>0.439</v>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="n">
+        <v>31.781255215535</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1702,7 +1706,9 @@
       <c r="H4" t="n">
         <v>0.469</v>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="n">
+        <v>34.0820996870785</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1735,7 +1741,9 @@
       <c r="H5" t="n">
         <v>0.442</v>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="n">
+        <v>38.8183409385794</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1768,7 +1776,9 @@
       <c r="H6" t="n">
         <v>0.404</v>
       </c>
-      <c r="I6" t="inlineStr"/>
+      <c r="I6" t="n">
+        <v>51.7928495263723</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1801,7 +1811,9 @@
       <c r="H7" t="n">
         <v>0.386</v>
       </c>
-      <c r="I7" t="inlineStr"/>
+      <c r="I7" t="n">
+        <v>52.5071622623698</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1834,7 +1846,9 @@
       <c r="H8" t="n">
         <v>0.381</v>
       </c>
-      <c r="I8" t="inlineStr"/>
+      <c r="I8" t="n">
+        <v>55.3644132056691</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1867,7 +1881,9 @@
       <c r="H9" t="n">
         <v>0.423</v>
       </c>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" t="n">
+        <v>62.1163594444336</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1900,7 +1916,9 @@
       <c r="H10" t="n">
         <v>0.399</v>
       </c>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" t="n">
+        <v>69.01064106942469</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1933,7 +1951,9 @@
       <c r="H11" t="n">
         <v>0.397</v>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="n">
+        <v>73.3196361410336</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1966,7 +1986,9 @@
       <c r="H12" t="n">
         <v>0.386</v>
       </c>
-      <c r="I12" t="inlineStr"/>
+      <c r="I12" t="n">
+        <v>79.302189298518</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1999,7 +2021,9 @@
       <c r="H13" t="n">
         <v>0.408</v>
       </c>
-      <c r="I13" t="inlineStr"/>
+      <c r="I13" t="n">
+        <v>83.14999999999999</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2032,7 +2056,9 @@
       <c r="H14" t="n">
         <v>0.395</v>
       </c>
-      <c r="I14" t="inlineStr"/>
+      <c r="I14" t="n">
+        <v>85.24166666666666</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2065,7 +2091,9 @@
       <c r="H15" t="n">
         <v>0.368</v>
       </c>
-      <c r="I15" t="inlineStr"/>
+      <c r="I15" t="n">
+        <v>92.80833333333334</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2098,7 +2126,9 @@
       <c r="H16" t="n">
         <v>0.393</v>
       </c>
-      <c r="I16" t="inlineStr"/>
+      <c r="I16" t="n">
+        <v>98.425</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2131,7 +2161,9 @@
       <c r="H17" t="n">
         <v>0.383</v>
       </c>
-      <c r="I17" t="inlineStr"/>
+      <c r="I17" t="n">
+        <v>104.9083333333334</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2164,7 +2196,9 @@
       <c r="H18" t="n">
         <v>0.324</v>
       </c>
-      <c r="I18" t="inlineStr"/>
+      <c r="I18" t="n">
+        <v>110.4833333333333</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2197,7 +2231,9 @@
       <c r="H19" t="n">
         <v>0.354</v>
       </c>
-      <c r="I19" t="inlineStr"/>
+      <c r="I19" t="n">
+        <v>115.15</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2230,7 +2266,9 @@
       <c r="H20" t="n">
         <v>0.366</v>
       </c>
-      <c r="I20" t="inlineStr"/>
+      <c r="I20" t="n">
+        <v>121.4833333333333</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2261,7 +2299,9 @@
         <v>5.9</v>
       </c>
       <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
+      <c r="I21" t="n">
+        <v>120.1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2295,7 +2335,7 @@
         <v>0.366</v>
       </c>
       <c r="I22" t="n">
-        <v>130.625</v>
+        <v>127.2333333333333</v>
       </c>
     </row>
     <row r="23">
@@ -2329,7 +2369,9 @@
       <c r="H23" t="n">
         <v>0.1207386683875913</v>
       </c>
-      <c r="I23" t="inlineStr"/>
+      <c r="I23" t="n">
+        <v>132.7916666666667</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2358,7 +2400,9 @@
         <v>63.2</v>
       </c>
       <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
+      <c r="I24" t="n">
+        <v>23.3563585414548</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2389,7 +2433,9 @@
       <c r="H25" t="n">
         <v>0.523</v>
       </c>
-      <c r="I25" t="inlineStr"/>
+      <c r="I25" t="n">
+        <v>31.781255215535</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2422,7 +2468,9 @@
       <c r="H26" t="n">
         <v>0.497</v>
       </c>
-      <c r="I26" t="inlineStr"/>
+      <c r="I26" t="n">
+        <v>34.0820996870785</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2455,7 +2503,9 @@
       <c r="H27" t="n">
         <v>0.468</v>
       </c>
-      <c r="I27" t="inlineStr"/>
+      <c r="I27" t="n">
+        <v>38.8183409385794</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2488,7 +2538,9 @@
       <c r="H28" t="n">
         <v>0.476</v>
       </c>
-      <c r="I28" t="inlineStr"/>
+      <c r="I28" t="n">
+        <v>51.7928495263723</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2521,7 +2573,9 @@
       <c r="H29" t="n">
         <v>0.434</v>
       </c>
-      <c r="I29" t="inlineStr"/>
+      <c r="I29" t="n">
+        <v>52.5071622623698</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2554,7 +2608,9 @@
       <c r="H30" t="n">
         <v>0.428</v>
       </c>
-      <c r="I30" t="inlineStr"/>
+      <c r="I30" t="n">
+        <v>55.3644132056691</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2587,7 +2643,9 @@
       <c r="H31" t="n">
         <v>0.433</v>
       </c>
-      <c r="I31" t="inlineStr"/>
+      <c r="I31" t="n">
+        <v>62.1163594444336</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2620,7 +2678,9 @@
       <c r="H32" t="n">
         <v>0.406</v>
       </c>
-      <c r="I32" t="inlineStr"/>
+      <c r="I32" t="n">
+        <v>69.01064106942469</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2653,7 +2713,9 @@
       <c r="H33" t="n">
         <v>0.429</v>
       </c>
-      <c r="I33" t="inlineStr"/>
+      <c r="I33" t="n">
+        <v>73.3196361410336</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2686,7 +2748,9 @@
       <c r="H34" t="n">
         <v>0.409</v>
       </c>
-      <c r="I34" t="inlineStr"/>
+      <c r="I34" t="n">
+        <v>79.302189298518</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2719,7 +2783,9 @@
       <c r="H35" t="n">
         <v>0.426</v>
       </c>
-      <c r="I35" t="inlineStr"/>
+      <c r="I35" t="n">
+        <v>83.14999999999999</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2752,7 +2818,9 @@
       <c r="H36" t="n">
         <v>0.387</v>
       </c>
-      <c r="I36" t="inlineStr"/>
+      <c r="I36" t="n">
+        <v>85.24166666666666</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2785,7 +2853,9 @@
       <c r="H37" t="n">
         <v>0.392</v>
       </c>
-      <c r="I37" t="inlineStr"/>
+      <c r="I37" t="n">
+        <v>92.80833333333334</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2818,7 +2888,9 @@
       <c r="H38" t="n">
         <v>0.408</v>
       </c>
-      <c r="I38" t="inlineStr"/>
+      <c r="I38" t="n">
+        <v>98.425</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2851,7 +2923,9 @@
       <c r="H39" t="n">
         <v>0.391</v>
       </c>
-      <c r="I39" t="inlineStr"/>
+      <c r="I39" t="n">
+        <v>104.9083333333334</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2884,7 +2958,9 @@
       <c r="H40" t="n">
         <v>0.365</v>
       </c>
-      <c r="I40" t="inlineStr"/>
+      <c r="I40" t="n">
+        <v>110.4833333333333</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2917,7 +2993,9 @@
       <c r="H41" t="n">
         <v>0.393</v>
       </c>
-      <c r="I41" t="inlineStr"/>
+      <c r="I41" t="n">
+        <v>115.15</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2950,7 +3028,9 @@
       <c r="H42" t="n">
         <v>0.354</v>
       </c>
-      <c r="I42" t="inlineStr"/>
+      <c r="I42" t="n">
+        <v>121.4833333333333</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2981,7 +3061,9 @@
         <v>12.7</v>
       </c>
       <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
+      <c r="I43" t="n">
+        <v>120.1</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3015,7 +3097,7 @@
         <v>0.359</v>
       </c>
       <c r="I44" t="n">
-        <v>123.475</v>
+        <v>127.2333333333333</v>
       </c>
     </row>
     <row r="45">
@@ -3049,7 +3131,9 @@
       <c r="H45" t="n">
         <v>0.05927313893117847</v>
       </c>
-      <c r="I45" t="inlineStr"/>
+      <c r="I45" t="n">
+        <v>132.7916666666667</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3078,7 +3162,9 @@
         <v>76.09999999999999</v>
       </c>
       <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
+      <c r="I46" t="n">
+        <v>23.3563585414548</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3109,7 +3195,9 @@
       <c r="H47" t="n">
         <v>0.612</v>
       </c>
-      <c r="I47" t="inlineStr"/>
+      <c r="I47" t="n">
+        <v>31.781255215535</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3142,7 +3230,9 @@
       <c r="H48" t="n">
         <v>0.505</v>
       </c>
-      <c r="I48" t="inlineStr"/>
+      <c r="I48" t="n">
+        <v>34.0820996870785</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3175,7 +3265,9 @@
       <c r="H49" t="n">
         <v>0.438</v>
       </c>
-      <c r="I49" t="inlineStr"/>
+      <c r="I49" t="n">
+        <v>38.8183409385794</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3208,7 +3300,9 @@
       <c r="H50" t="n">
         <v>0.464</v>
       </c>
-      <c r="I50" t="inlineStr"/>
+      <c r="I50" t="n">
+        <v>51.7928495263723</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3241,7 +3335,9 @@
       <c r="H51" t="n">
         <v>0.414</v>
       </c>
-      <c r="I51" t="inlineStr"/>
+      <c r="I51" t="n">
+        <v>52.5071622623698</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3274,7 +3370,9 @@
       <c r="H52" t="n">
         <v>0.407</v>
       </c>
-      <c r="I52" t="inlineStr"/>
+      <c r="I52" t="n">
+        <v>55.3644132056691</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3307,7 +3405,9 @@
       <c r="H53" t="n">
         <v>0.451</v>
       </c>
-      <c r="I53" t="inlineStr"/>
+      <c r="I53" t="n">
+        <v>62.1163594444336</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3340,7 +3440,9 @@
       <c r="H54" t="n">
         <v>0.442</v>
       </c>
-      <c r="I54" t="inlineStr"/>
+      <c r="I54" t="n">
+        <v>69.01064106942469</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3373,7 +3475,9 @@
       <c r="H55" t="n">
         <v>0.442</v>
       </c>
-      <c r="I55" t="inlineStr"/>
+      <c r="I55" t="n">
+        <v>73.3196361410336</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3406,7 +3510,9 @@
       <c r="H56" t="n">
         <v>0.424</v>
       </c>
-      <c r="I56" t="inlineStr"/>
+      <c r="I56" t="n">
+        <v>79.302189298518</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3439,7 +3545,9 @@
       <c r="H57" t="n">
         <v>0.444</v>
       </c>
-      <c r="I57" t="inlineStr"/>
+      <c r="I57" t="n">
+        <v>83.14999999999999</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3472,7 +3580,9 @@
       <c r="H58" t="n">
         <v>0.416</v>
       </c>
-      <c r="I58" t="inlineStr"/>
+      <c r="I58" t="n">
+        <v>85.24166666666666</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3505,7 +3615,9 @@
       <c r="H59" t="n">
         <v>0.405</v>
       </c>
-      <c r="I59" t="inlineStr"/>
+      <c r="I59" t="n">
+        <v>92.80833333333334</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3538,7 +3650,9 @@
       <c r="H60" t="n">
         <v>0.428</v>
       </c>
-      <c r="I60" t="inlineStr"/>
+      <c r="I60" t="n">
+        <v>98.425</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3571,7 +3685,9 @@
       <c r="H61" t="n">
         <v>0.41</v>
       </c>
-      <c r="I61" t="inlineStr"/>
+      <c r="I61" t="n">
+        <v>104.9083333333334</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3604,7 +3720,9 @@
       <c r="H62" t="n">
         <v>0.393</v>
       </c>
-      <c r="I62" t="inlineStr"/>
+      <c r="I62" t="n">
+        <v>110.4833333333333</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3637,7 +3755,9 @@
       <c r="H63" t="n">
         <v>0.389</v>
       </c>
-      <c r="I63" t="inlineStr"/>
+      <c r="I63" t="n">
+        <v>115.15</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3670,7 +3790,9 @@
       <c r="H64" t="n">
         <v>0.378</v>
       </c>
-      <c r="I64" t="inlineStr"/>
+      <c r="I64" t="n">
+        <v>121.4833333333333</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3701,7 +3823,9 @@
         <v>21.2</v>
       </c>
       <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
+      <c r="I65" t="n">
+        <v>120.1</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3735,7 +3859,7 @@
         <v>0.385</v>
       </c>
       <c r="I66" t="n">
-        <v>125.875</v>
+        <v>127.2333333333333</v>
       </c>
     </row>
     <row r="67">
@@ -3769,7 +3893,9 @@
       <c r="H67" t="n">
         <v>0.08187821936581452</v>
       </c>
-      <c r="I67" t="inlineStr"/>
+      <c r="I67" t="n">
+        <v>132.7916666666667</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3798,7 +3924,9 @@
         <v>44.9</v>
       </c>
       <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr"/>
+      <c r="I68" t="n">
+        <v>23.3563585414548</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3829,7 +3957,9 @@
       <c r="H69" t="n">
         <v>0.506</v>
       </c>
-      <c r="I69" t="inlineStr"/>
+      <c r="I69" t="n">
+        <v>31.781255215535</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3862,7 +3992,9 @@
       <c r="H70" t="n">
         <v>0.5580000000000001</v>
       </c>
-      <c r="I70" t="inlineStr"/>
+      <c r="I70" t="n">
+        <v>34.0820996870785</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3895,7 +4027,9 @@
       <c r="H71" t="n">
         <v>0.472</v>
       </c>
-      <c r="I71" t="inlineStr"/>
+      <c r="I71" t="n">
+        <v>38.8183409385794</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3928,7 +4062,9 @@
       <c r="H72" t="n">
         <v>0.438</v>
       </c>
-      <c r="I72" t="inlineStr"/>
+      <c r="I72" t="n">
+        <v>51.7928495263723</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3961,7 +4097,9 @@
       <c r="H73" t="n">
         <v>0.403</v>
       </c>
-      <c r="I73" t="inlineStr"/>
+      <c r="I73" t="n">
+        <v>52.5071622623698</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3994,7 +4132,9 @@
       <c r="H74" t="n">
         <v>0.396</v>
       </c>
-      <c r="I74" t="inlineStr"/>
+      <c r="I74" t="n">
+        <v>55.3644132056691</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4027,7 +4167,9 @@
       <c r="H75" t="n">
         <v>0.397</v>
       </c>
-      <c r="I75" t="inlineStr"/>
+      <c r="I75" t="n">
+        <v>62.1163594444336</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4060,7 +4202,9 @@
       <c r="H76" t="n">
         <v>0.399</v>
       </c>
-      <c r="I76" t="inlineStr"/>
+      <c r="I76" t="n">
+        <v>69.01064106942469</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4093,7 +4237,9 @@
       <c r="H77" t="n">
         <v>0.371</v>
       </c>
-      <c r="I77" t="inlineStr"/>
+      <c r="I77" t="n">
+        <v>73.3196361410336</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4126,7 +4272,9 @@
       <c r="H78" t="n">
         <v>0.399</v>
       </c>
-      <c r="I78" t="inlineStr"/>
+      <c r="I78" t="n">
+        <v>79.302189298518</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4159,7 +4307,9 @@
       <c r="H79" t="n">
         <v>0.386</v>
       </c>
-      <c r="I79" t="inlineStr"/>
+      <c r="I79" t="n">
+        <v>83.14999999999999</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4192,7 +4342,9 @@
       <c r="H80" t="n">
         <v>0.352</v>
       </c>
-      <c r="I80" t="inlineStr"/>
+      <c r="I80" t="n">
+        <v>85.24166666666666</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4225,7 +4377,9 @@
       <c r="H81" t="n">
         <v>0.38</v>
       </c>
-      <c r="I81" t="inlineStr"/>
+      <c r="I81" t="n">
+        <v>92.80833333333334</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4258,7 +4412,9 @@
       <c r="H82" t="n">
         <v>0.411</v>
       </c>
-      <c r="I82" t="inlineStr"/>
+      <c r="I82" t="n">
+        <v>98.425</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4291,7 +4447,9 @@
       <c r="H83" t="n">
         <v>0.355</v>
       </c>
-      <c r="I83" t="inlineStr"/>
+      <c r="I83" t="n">
+        <v>104.9083333333334</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4324,7 +4482,9 @@
       <c r="H84" t="n">
         <v>0.316</v>
       </c>
-      <c r="I84" t="inlineStr"/>
+      <c r="I84" t="n">
+        <v>110.4833333333333</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4357,7 +4517,9 @@
       <c r="H85" t="n">
         <v>0.337</v>
       </c>
-      <c r="I85" t="inlineStr"/>
+      <c r="I85" t="n">
+        <v>115.15</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4390,7 +4552,9 @@
       <c r="H86" t="n">
         <v>0.383</v>
       </c>
-      <c r="I86" t="inlineStr"/>
+      <c r="I86" t="n">
+        <v>121.4833333333333</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4421,7 +4585,9 @@
         <v>6.1</v>
       </c>
       <c r="H87" t="inlineStr"/>
-      <c r="I87" t="inlineStr"/>
+      <c r="I87" t="n">
+        <v>120.1</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4455,7 +4621,7 @@
         <v>0.37</v>
       </c>
       <c r="I88" t="n">
-        <v>124.1916666666667</v>
+        <v>127.2333333333333</v>
       </c>
     </row>
     <row r="89">
@@ -4489,7 +4655,9 @@
       <c r="H89" t="n">
         <v>0.05523604590505982</v>
       </c>
-      <c r="I89" t="inlineStr"/>
+      <c r="I89" t="n">
+        <v>132.7916666666667</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4518,7 +4686,9 @@
         <v>44.8</v>
       </c>
       <c r="H90" t="inlineStr"/>
-      <c r="I90" t="inlineStr"/>
+      <c r="I90" t="n">
+        <v>23.3563585414548</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4549,7 +4719,9 @@
       <c r="H91" t="n">
         <v>0.465</v>
       </c>
-      <c r="I91" t="inlineStr"/>
+      <c r="I91" t="n">
+        <v>31.781255215535</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4582,7 +4754,9 @@
       <c r="H92" t="n">
         <v>0.49</v>
       </c>
-      <c r="I92" t="inlineStr"/>
+      <c r="I92" t="n">
+        <v>34.0820996870785</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4615,7 +4789,9 @@
       <c r="H93" t="n">
         <v>0.432</v>
       </c>
-      <c r="I93" t="inlineStr"/>
+      <c r="I93" t="n">
+        <v>38.8183409385794</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4648,7 +4824,9 @@
       <c r="H94" t="n">
         <v>0.422</v>
       </c>
-      <c r="I94" t="inlineStr"/>
+      <c r="I94" t="n">
+        <v>51.7928495263723</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4681,7 +4859,9 @@
       <c r="H95" t="n">
         <v>0.431</v>
       </c>
-      <c r="I95" t="inlineStr"/>
+      <c r="I95" t="n">
+        <v>52.5071622623698</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4714,7 +4894,9 @@
       <c r="H96" t="n">
         <v>0.366</v>
       </c>
-      <c r="I96" t="inlineStr"/>
+      <c r="I96" t="n">
+        <v>55.3644132056691</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -4747,7 +4929,9 @@
       <c r="H97" t="n">
         <v>0.406</v>
       </c>
-      <c r="I97" t="inlineStr"/>
+      <c r="I97" t="n">
+        <v>62.1163594444336</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -4780,7 +4964,9 @@
       <c r="H98" t="n">
         <v>0.384</v>
       </c>
-      <c r="I98" t="inlineStr"/>
+      <c r="I98" t="n">
+        <v>69.01064106942469</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -4813,7 +4999,9 @@
       <c r="H99" t="n">
         <v>0.408</v>
       </c>
-      <c r="I99" t="inlineStr"/>
+      <c r="I99" t="n">
+        <v>73.3196361410336</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -4846,7 +5034,9 @@
       <c r="H100" t="n">
         <v>0.392</v>
       </c>
-      <c r="I100" t="inlineStr"/>
+      <c r="I100" t="n">
+        <v>79.302189298518</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -4879,7 +5069,9 @@
       <c r="H101" t="n">
         <v>0.401</v>
       </c>
-      <c r="I101" t="inlineStr"/>
+      <c r="I101" t="n">
+        <v>83.14999999999999</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -4912,7 +5104,9 @@
       <c r="H102" t="n">
         <v>0.38</v>
       </c>
-      <c r="I102" t="inlineStr"/>
+      <c r="I102" t="n">
+        <v>85.24166666666666</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -4945,7 +5139,9 @@
       <c r="H103" t="n">
         <v>0.385</v>
       </c>
-      <c r="I103" t="inlineStr"/>
+      <c r="I103" t="n">
+        <v>92.80833333333334</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -4978,7 +5174,9 @@
       <c r="H104" t="n">
         <v>0.372</v>
       </c>
-      <c r="I104" t="inlineStr"/>
+      <c r="I104" t="n">
+        <v>98.425</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -5011,7 +5209,9 @@
       <c r="H105" t="n">
         <v>0.382</v>
       </c>
-      <c r="I105" t="inlineStr"/>
+      <c r="I105" t="n">
+        <v>104.9083333333334</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -5044,7 +5244,9 @@
       <c r="H106" t="n">
         <v>0.361</v>
       </c>
-      <c r="I106" t="inlineStr"/>
+      <c r="I106" t="n">
+        <v>110.4833333333333</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -5077,7 +5279,9 @@
       <c r="H107" t="n">
         <v>0.38</v>
       </c>
-      <c r="I107" t="inlineStr"/>
+      <c r="I107" t="n">
+        <v>115.15</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -5110,7 +5314,9 @@
       <c r="H108" t="n">
         <v>0.391</v>
       </c>
-      <c r="I108" t="inlineStr"/>
+      <c r="I108" t="n">
+        <v>121.4833333333333</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -5141,7 +5347,9 @@
         <v>6.5</v>
       </c>
       <c r="H109" t="inlineStr"/>
-      <c r="I109" t="inlineStr"/>
+      <c r="I109" t="n">
+        <v>120.1</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -5174,7 +5382,9 @@
       <c r="H110" t="n">
         <v>0.369</v>
       </c>
-      <c r="I110" t="inlineStr"/>
+      <c r="I110" t="n">
+        <v>127.2333333333333</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -5207,7 +5417,9 @@
       <c r="H111" t="n">
         <v>0.1261501222305634</v>
       </c>
-      <c r="I111" t="inlineStr"/>
+      <c r="I111" t="n">
+        <v>132.7916666666667</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -5236,7 +5448,9 @@
         <v>43.2</v>
       </c>
       <c r="H112" t="inlineStr"/>
-      <c r="I112" t="inlineStr"/>
+      <c r="I112" t="n">
+        <v>23.3563585414548</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -5267,7 +5481,9 @@
       <c r="H113" t="n">
         <v>0.445</v>
       </c>
-      <c r="I113" t="inlineStr"/>
+      <c r="I113" t="n">
+        <v>31.781255215535</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -5300,7 +5516,9 @@
       <c r="H114" t="n">
         <v>0.384</v>
       </c>
-      <c r="I114" t="inlineStr"/>
+      <c r="I114" t="n">
+        <v>34.0820996870785</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -5333,7 +5551,9 @@
       <c r="H115" t="n">
         <v>0.478</v>
       </c>
-      <c r="I115" t="inlineStr"/>
+      <c r="I115" t="n">
+        <v>38.8183409385794</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -5366,7 +5586,9 @@
       <c r="H116" t="n">
         <v>0.416</v>
       </c>
-      <c r="I116" t="inlineStr"/>
+      <c r="I116" t="n">
+        <v>51.7928495263723</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -5399,7 +5621,9 @@
       <c r="H117" t="n">
         <v>0.372</v>
       </c>
-      <c r="I117" t="inlineStr"/>
+      <c r="I117" t="n">
+        <v>52.5071622623698</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -5432,7 +5656,9 @@
       <c r="H118" t="n">
         <v>0.35</v>
       </c>
-      <c r="I118" t="inlineStr"/>
+      <c r="I118" t="n">
+        <v>55.3644132056691</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -5465,7 +5691,9 @@
       <c r="H119" t="n">
         <v>0.369</v>
       </c>
-      <c r="I119" t="inlineStr"/>
+      <c r="I119" t="n">
+        <v>62.1163594444336</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -5498,7 +5726,9 @@
       <c r="H120" t="n">
         <v>0.373</v>
       </c>
-      <c r="I120" t="inlineStr"/>
+      <c r="I120" t="n">
+        <v>69.01064106942469</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -5531,7 +5761,9 @@
       <c r="H121" t="n">
         <v>0.359</v>
       </c>
-      <c r="I121" t="inlineStr"/>
+      <c r="I121" t="n">
+        <v>73.3196361410336</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -5564,7 +5796,9 @@
       <c r="H122" t="n">
         <v>0.332</v>
       </c>
-      <c r="I122" t="inlineStr"/>
+      <c r="I122" t="n">
+        <v>79.302189298518</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -5597,7 +5831,9 @@
       <c r="H123" t="n">
         <v>0.404</v>
       </c>
-      <c r="I123" t="inlineStr"/>
+      <c r="I123" t="n">
+        <v>83.14999999999999</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -5630,7 +5866,9 @@
       <c r="H124" t="n">
         <v>0.389</v>
       </c>
-      <c r="I124" t="inlineStr"/>
+      <c r="I124" t="n">
+        <v>85.24166666666666</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -5663,7 +5901,9 @@
       <c r="H125" t="n">
         <v>0.38</v>
       </c>
-      <c r="I125" t="inlineStr"/>
+      <c r="I125" t="n">
+        <v>92.80833333333334</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -5696,7 +5936,9 @@
       <c r="H126" t="n">
         <v>0.382</v>
       </c>
-      <c r="I126" t="inlineStr"/>
+      <c r="I126" t="n">
+        <v>98.425</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -5729,7 +5971,9 @@
       <c r="H127" t="n">
         <v>0.354</v>
       </c>
-      <c r="I127" t="inlineStr"/>
+      <c r="I127" t="n">
+        <v>104.9083333333334</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -5762,7 +6006,9 @@
       <c r="H128" t="n">
         <v>0.36</v>
       </c>
-      <c r="I128" t="inlineStr"/>
+      <c r="I128" t="n">
+        <v>110.4833333333333</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -5795,7 +6041,9 @@
       <c r="H129" t="n">
         <v>0.324</v>
       </c>
-      <c r="I129" t="inlineStr"/>
+      <c r="I129" t="n">
+        <v>115.15</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -5828,7 +6076,9 @@
       <c r="H130" t="n">
         <v>0.33</v>
       </c>
-      <c r="I130" t="inlineStr"/>
+      <c r="I130" t="n">
+        <v>121.4833333333333</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -5859,7 +6109,9 @@
         <v>8.800000000000001</v>
       </c>
       <c r="H131" t="inlineStr"/>
-      <c r="I131" t="inlineStr"/>
+      <c r="I131" t="n">
+        <v>120.1</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -5893,7 +6145,7 @@
         <v>0.308</v>
       </c>
       <c r="I132" t="n">
-        <v>124.6833333333333</v>
+        <v>127.2333333333333</v>
       </c>
     </row>
     <row r="133">
@@ -5927,7 +6179,9 @@
       <c r="H133" t="n">
         <v>0.07221019055698719</v>
       </c>
-      <c r="I133" t="inlineStr"/>
+      <c r="I133" t="n">
+        <v>132.7916666666667</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -5956,7 +6210,9 @@
         <v>48.6</v>
       </c>
       <c r="H134" t="inlineStr"/>
-      <c r="I134" t="inlineStr"/>
+      <c r="I134" t="n">
+        <v>23.3563585414548</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -5987,7 +6243,9 @@
       <c r="H135" t="n">
         <v>0.452</v>
       </c>
-      <c r="I135" t="inlineStr"/>
+      <c r="I135" t="n">
+        <v>31.781255215535</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -6020,7 +6278,9 @@
       <c r="H136" t="n">
         <v>0.525</v>
       </c>
-      <c r="I136" t="inlineStr"/>
+      <c r="I136" t="n">
+        <v>34.0820996870785</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -6053,7 +6313,9 @@
       <c r="H137" t="n">
         <v>0.447</v>
       </c>
-      <c r="I137" t="inlineStr"/>
+      <c r="I137" t="n">
+        <v>38.8183409385794</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -6086,7 +6348,9 @@
       <c r="H138" t="n">
         <v>0.428</v>
       </c>
-      <c r="I138" t="inlineStr"/>
+      <c r="I138" t="n">
+        <v>51.7928495263723</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -6119,7 +6383,9 @@
       <c r="H139" t="n">
         <v>0.41</v>
       </c>
-      <c r="I139" t="inlineStr"/>
+      <c r="I139" t="n">
+        <v>52.5071622623698</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -6152,7 +6418,9 @@
       <c r="H140" t="n">
         <v>0.421</v>
       </c>
-      <c r="I140" t="inlineStr"/>
+      <c r="I140" t="n">
+        <v>55.3644132056691</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -6185,7 +6453,9 @@
       <c r="H141" t="n">
         <v>0.399</v>
       </c>
-      <c r="I141" t="inlineStr"/>
+      <c r="I141" t="n">
+        <v>62.1163594444336</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -6218,7 +6488,9 @@
       <c r="H142" t="n">
         <v>0.397</v>
       </c>
-      <c r="I142" t="inlineStr"/>
+      <c r="I142" t="n">
+        <v>69.01064106942469</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -6251,7 +6523,9 @@
       <c r="H143" t="n">
         <v>0.381</v>
       </c>
-      <c r="I143" t="inlineStr"/>
+      <c r="I143" t="n">
+        <v>73.3196361410336</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -6284,7 +6558,9 @@
       <c r="H144" t="n">
         <v>0.387</v>
       </c>
-      <c r="I144" t="inlineStr"/>
+      <c r="I144" t="n">
+        <v>79.302189298518</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -6317,7 +6593,9 @@
       <c r="H145" t="n">
         <v>0.417</v>
       </c>
-      <c r="I145" t="inlineStr"/>
+      <c r="I145" t="n">
+        <v>83.14999999999999</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -6350,7 +6628,9 @@
       <c r="H146" t="n">
         <v>0.393</v>
       </c>
-      <c r="I146" t="inlineStr"/>
+      <c r="I146" t="n">
+        <v>85.24166666666666</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -6383,7 +6663,9 @@
       <c r="H147" t="n">
         <v>0.399</v>
       </c>
-      <c r="I147" t="inlineStr"/>
+      <c r="I147" t="n">
+        <v>92.80833333333334</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -6416,7 +6698,9 @@
       <c r="H148" t="n">
         <v>0.4</v>
       </c>
-      <c r="I148" t="inlineStr"/>
+      <c r="I148" t="n">
+        <v>98.425</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -6449,7 +6733,9 @@
       <c r="H149" t="n">
         <v>0.417</v>
       </c>
-      <c r="I149" t="inlineStr"/>
+      <c r="I149" t="n">
+        <v>104.9083333333334</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -6482,7 +6768,9 @@
       <c r="H150" t="n">
         <v>0.366</v>
       </c>
-      <c r="I150" t="inlineStr"/>
+      <c r="I150" t="n">
+        <v>110.4833333333333</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -6515,7 +6803,9 @@
       <c r="H151" t="n">
         <v>0.362</v>
       </c>
-      <c r="I151" t="inlineStr"/>
+      <c r="I151" t="n">
+        <v>115.15</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -6548,7 +6838,9 @@
       <c r="H152" t="n">
         <v>0.377</v>
       </c>
-      <c r="I152" t="inlineStr"/>
+      <c r="I152" t="n">
+        <v>121.4833333333333</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -6579,7 +6871,9 @@
         <v>11.4</v>
       </c>
       <c r="H153" t="inlineStr"/>
-      <c r="I153" t="inlineStr"/>
+      <c r="I153" t="n">
+        <v>120.1</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -6613,7 +6907,7 @@
         <v>0.368</v>
       </c>
       <c r="I154" t="n">
-        <v>122.95</v>
+        <v>127.2333333333333</v>
       </c>
     </row>
     <row r="155">
@@ -6647,7 +6941,9 @@
       <c r="H155" t="n">
         <v>0.07434198217656229</v>
       </c>
-      <c r="I155" t="inlineStr"/>
+      <c r="I155" t="n">
+        <v>132.7916666666667</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -6676,7 +6972,9 @@
         <v>73.90000000000001</v>
       </c>
       <c r="H156" t="inlineStr"/>
-      <c r="I156" t="inlineStr"/>
+      <c r="I156" t="n">
+        <v>23.3563585414548</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -6707,7 +7005,9 @@
       <c r="H157" t="n">
         <v>0.425</v>
       </c>
-      <c r="I157" t="inlineStr"/>
+      <c r="I157" t="n">
+        <v>31.781255215535</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -6740,7 +7040,9 @@
       <c r="H158" t="n">
         <v>0.498</v>
       </c>
-      <c r="I158" t="inlineStr"/>
+      <c r="I158" t="n">
+        <v>34.0820996870785</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -6773,7 +7075,9 @@
       <c r="H159" t="n">
         <v>0.44</v>
       </c>
-      <c r="I159" t="inlineStr"/>
+      <c r="I159" t="n">
+        <v>38.8183409385794</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -6806,7 +7110,9 @@
       <c r="H160" t="n">
         <v>0.459</v>
       </c>
-      <c r="I160" t="inlineStr"/>
+      <c r="I160" t="n">
+        <v>51.7928495263723</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -6839,7 +7145,9 @@
       <c r="H161" t="n">
         <v>0.408</v>
       </c>
-      <c r="I161" t="inlineStr"/>
+      <c r="I161" t="n">
+        <v>52.5071622623698</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -6872,7 +7180,9 @@
       <c r="H162" t="n">
         <v>0.377</v>
       </c>
-      <c r="I162" t="inlineStr"/>
+      <c r="I162" t="n">
+        <v>55.3644132056691</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -6905,7 +7215,9 @@
       <c r="H163" t="n">
         <v>0.415</v>
       </c>
-      <c r="I163" t="inlineStr"/>
+      <c r="I163" t="n">
+        <v>62.1163594444336</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -6938,7 +7250,9 @@
       <c r="H164" t="n">
         <v>0.379</v>
       </c>
-      <c r="I164" t="inlineStr"/>
+      <c r="I164" t="n">
+        <v>69.01064106942469</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -6971,7 +7285,9 @@
       <c r="H165" t="n">
         <v>0.412</v>
       </c>
-      <c r="I165" t="inlineStr"/>
+      <c r="I165" t="n">
+        <v>73.3196361410336</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -7004,7 +7320,9 @@
       <c r="H166" t="n">
         <v>0.394</v>
       </c>
-      <c r="I166" t="inlineStr"/>
+      <c r="I166" t="n">
+        <v>79.302189298518</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -7037,7 +7355,9 @@
       <c r="H167" t="n">
         <v>0.437</v>
       </c>
-      <c r="I167" t="inlineStr"/>
+      <c r="I167" t="n">
+        <v>83.14999999999999</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -7070,7 +7390,9 @@
       <c r="H168" t="n">
         <v>0.423</v>
       </c>
-      <c r="I168" t="inlineStr"/>
+      <c r="I168" t="n">
+        <v>85.24166666666666</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -7103,7 +7425,9 @@
       <c r="H169" t="n">
         <v>0.454</v>
       </c>
-      <c r="I169" t="inlineStr"/>
+      <c r="I169" t="n">
+        <v>92.80833333333334</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -7136,7 +7460,9 @@
       <c r="H170" t="n">
         <v>0.434</v>
       </c>
-      <c r="I170" t="inlineStr"/>
+      <c r="I170" t="n">
+        <v>98.425</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -7169,7 +7495,9 @@
       <c r="H171" t="n">
         <v>0.455</v>
       </c>
-      <c r="I171" t="inlineStr"/>
+      <c r="I171" t="n">
+        <v>104.9083333333334</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -7202,7 +7530,9 @@
       <c r="H172" t="n">
         <v>0.346</v>
       </c>
-      <c r="I172" t="inlineStr"/>
+      <c r="I172" t="n">
+        <v>110.4833333333333</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -7235,7 +7565,9 @@
       <c r="H173" t="n">
         <v>0.327</v>
       </c>
-      <c r="I173" t="inlineStr"/>
+      <c r="I173" t="n">
+        <v>115.15</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -7268,7 +7600,9 @@
       <c r="H174" t="n">
         <v>0.334</v>
       </c>
-      <c r="I174" t="inlineStr"/>
+      <c r="I174" t="n">
+        <v>121.4833333333333</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -7299,7 +7633,9 @@
         <v>9.9</v>
       </c>
       <c r="H175" t="inlineStr"/>
-      <c r="I175" t="inlineStr"/>
+      <c r="I175" t="n">
+        <v>120.1</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -7333,7 +7669,7 @@
         <v>0.336</v>
       </c>
       <c r="I176" t="n">
-        <v>120.1666666666667</v>
+        <v>127.2333333333333</v>
       </c>
     </row>
     <row r="177">
@@ -7367,7 +7703,9 @@
       <c r="H177" t="n">
         <v>0.01578437942074307</v>
       </c>
-      <c r="I177" t="inlineStr"/>
+      <c r="I177" t="n">
+        <v>132.7916666666667</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -7396,7 +7734,9 @@
         <v>43.7</v>
       </c>
       <c r="H178" t="inlineStr"/>
-      <c r="I178" t="inlineStr"/>
+      <c r="I178" t="n">
+        <v>23.3563585414548</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -7427,7 +7767,9 @@
       <c r="H179" t="n">
         <v>0.597</v>
       </c>
-      <c r="I179" t="inlineStr"/>
+      <c r="I179" t="n">
+        <v>31.781255215535</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -7460,7 +7802,9 @@
       <c r="H180" t="n">
         <v>0.608</v>
       </c>
-      <c r="I180" t="inlineStr"/>
+      <c r="I180" t="n">
+        <v>34.0820996870785</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -7493,7 +7837,9 @@
       <c r="H181" t="n">
         <v>0.492</v>
       </c>
-      <c r="I181" t="inlineStr"/>
+      <c r="I181" t="n">
+        <v>38.8183409385794</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -7526,7 +7872,9 @@
       <c r="H182" t="n">
         <v>0.452</v>
       </c>
-      <c r="I182" t="inlineStr"/>
+      <c r="I182" t="n">
+        <v>51.7928495263723</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -7559,7 +7907,9 @@
       <c r="H183" t="n">
         <v>0.422</v>
       </c>
-      <c r="I183" t="inlineStr"/>
+      <c r="I183" t="n">
+        <v>52.5071622623698</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -7592,7 +7942,9 @@
       <c r="H184" t="n">
         <v>0.406</v>
       </c>
-      <c r="I184" t="inlineStr"/>
+      <c r="I184" t="n">
+        <v>55.3644132056691</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -7625,7 +7977,9 @@
       <c r="H185" t="n">
         <v>0.412</v>
       </c>
-      <c r="I185" t="inlineStr"/>
+      <c r="I185" t="n">
+        <v>62.1163594444336</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -7658,7 +8012,9 @@
       <c r="H186" t="n">
         <v>0.405</v>
       </c>
-      <c r="I186" t="inlineStr"/>
+      <c r="I186" t="n">
+        <v>69.01064106942469</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -7691,7 +8047,9 @@
       <c r="H187" t="n">
         <v>0.398</v>
       </c>
-      <c r="I187" t="inlineStr"/>
+      <c r="I187" t="n">
+        <v>73.3196361410336</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -7724,7 +8082,9 @@
       <c r="H188" t="n">
         <v>0.399</v>
       </c>
-      <c r="I188" t="inlineStr"/>
+      <c r="I188" t="n">
+        <v>79.302189298518</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -7757,7 +8117,9 @@
       <c r="H189" t="n">
         <v>0.435</v>
       </c>
-      <c r="I189" t="inlineStr"/>
+      <c r="I189" t="n">
+        <v>83.14999999999999</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -7790,7 +8152,9 @@
       <c r="H190" t="n">
         <v>0.398</v>
       </c>
-      <c r="I190" t="inlineStr"/>
+      <c r="I190" t="n">
+        <v>85.24166666666666</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -7823,7 +8187,9 @@
       <c r="H191" t="n">
         <v>0.411</v>
       </c>
-      <c r="I191" t="inlineStr"/>
+      <c r="I191" t="n">
+        <v>92.80833333333334</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -7856,7 +8222,9 @@
       <c r="H192" t="n">
         <v>0.419</v>
       </c>
-      <c r="I192" t="inlineStr"/>
+      <c r="I192" t="n">
+        <v>98.425</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -7889,7 +8257,9 @@
       <c r="H193" t="n">
         <v>0.37</v>
       </c>
-      <c r="I193" t="inlineStr"/>
+      <c r="I193" t="n">
+        <v>104.9083333333334</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -7922,7 +8292,9 @@
       <c r="H194" t="n">
         <v>0.364</v>
       </c>
-      <c r="I194" t="inlineStr"/>
+      <c r="I194" t="n">
+        <v>110.4833333333333</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -7955,7 +8327,9 @@
       <c r="H195" t="n">
         <v>0.356</v>
       </c>
-      <c r="I195" t="inlineStr"/>
+      <c r="I195" t="n">
+        <v>115.15</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -7988,7 +8362,9 @@
       <c r="H196" t="n">
         <v>0.359</v>
       </c>
-      <c r="I196" t="inlineStr"/>
+      <c r="I196" t="n">
+        <v>121.4833333333333</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -8019,7 +8395,9 @@
         <v>3.3</v>
       </c>
       <c r="H197" t="inlineStr"/>
-      <c r="I197" t="inlineStr"/>
+      <c r="I197" t="n">
+        <v>120.1</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -8052,7 +8430,9 @@
       <c r="H198" t="n">
         <v>0.371</v>
       </c>
-      <c r="I198" t="inlineStr"/>
+      <c r="I198" t="n">
+        <v>127.2333333333333</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -8085,7 +8465,9 @@
       <c r="H199" t="n">
         <v>0.08470763376623558</v>
       </c>
-      <c r="I199" t="inlineStr"/>
+      <c r="I199" t="n">
+        <v>132.7916666666667</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -8116,7 +8498,9 @@
         <v>58.3</v>
       </c>
       <c r="H200" t="inlineStr"/>
-      <c r="I200" t="inlineStr"/>
+      <c r="I200" t="n">
+        <v>34.0820996870785</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -8149,7 +8533,9 @@
       <c r="H201" t="n">
         <v>0.49</v>
       </c>
-      <c r="I201" t="inlineStr"/>
+      <c r="I201" t="n">
+        <v>38.8183409385794</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -8182,7 +8568,9 @@
       <c r="H202" t="n">
         <v>0.491</v>
       </c>
-      <c r="I202" t="inlineStr"/>
+      <c r="I202" t="n">
+        <v>51.7928495263723</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -8215,7 +8603,9 @@
       <c r="H203" t="n">
         <v>0.467</v>
       </c>
-      <c r="I203" t="inlineStr"/>
+      <c r="I203" t="n">
+        <v>52.5071622623698</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -8248,7 +8638,9 @@
       <c r="H204" t="n">
         <v>0.459</v>
       </c>
-      <c r="I204" t="inlineStr"/>
+      <c r="I204" t="n">
+        <v>55.3644132056691</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -8281,7 +8673,9 @@
       <c r="H205" t="n">
         <v>0.468</v>
       </c>
-      <c r="I205" t="inlineStr"/>
+      <c r="I205" t="n">
+        <v>62.1163594444336</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -8314,7 +8708,9 @@
       <c r="H206" t="n">
         <v>0.448</v>
       </c>
-      <c r="I206" t="inlineStr"/>
+      <c r="I206" t="n">
+        <v>69.01064106942469</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -8347,7 +8743,9 @@
       <c r="H207" t="n">
         <v>0.454</v>
       </c>
-      <c r="I207" t="inlineStr"/>
+      <c r="I207" t="n">
+        <v>73.3196361410336</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -8380,7 +8778,9 @@
       <c r="H208" t="n">
         <v>0.448</v>
       </c>
-      <c r="I208" t="inlineStr"/>
+      <c r="I208" t="n">
+        <v>79.302189298518</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -8413,7 +8813,9 @@
       <c r="H209" t="n">
         <v>0.465</v>
       </c>
-      <c r="I209" t="inlineStr"/>
+      <c r="I209" t="n">
+        <v>83.14999999999999</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -8446,7 +8848,9 @@
       <c r="H210" t="n">
         <v>0.477</v>
       </c>
-      <c r="I210" t="inlineStr"/>
+      <c r="I210" t="n">
+        <v>85.24166666666666</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -8479,7 +8883,9 @@
       <c r="H211" t="n">
         <v>0.451</v>
       </c>
-      <c r="I211" t="inlineStr"/>
+      <c r="I211" t="n">
+        <v>92.80833333333334</v>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -8512,7 +8918,9 @@
       <c r="H212" t="n">
         <v>0.454</v>
       </c>
-      <c r="I212" t="inlineStr"/>
+      <c r="I212" t="n">
+        <v>98.425</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -8545,7 +8953,9 @@
       <c r="H213" t="n">
         <v>0.427</v>
       </c>
-      <c r="I213" t="inlineStr"/>
+      <c r="I213" t="n">
+        <v>104.9083333333334</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -8578,7 +8988,9 @@
       <c r="H214" t="n">
         <v>0.387</v>
       </c>
-      <c r="I214" t="inlineStr"/>
+      <c r="I214" t="n">
+        <v>110.4833333333333</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -8611,7 +9023,9 @@
       <c r="H215" t="n">
         <v>0.402</v>
       </c>
-      <c r="I215" t="inlineStr"/>
+      <c r="I215" t="n">
+        <v>115.15</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -8644,7 +9058,9 @@
       <c r="H216" t="n">
         <v>0.397</v>
       </c>
-      <c r="I216" t="inlineStr"/>
+      <c r="I216" t="n">
+        <v>121.4833333333333</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -8675,7 +9091,9 @@
         <v>25.3</v>
       </c>
       <c r="H217" t="inlineStr"/>
-      <c r="I217" t="inlineStr"/>
+      <c r="I217" t="n">
+        <v>120.1</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -8709,7 +9127,7 @@
         <v>0.395</v>
       </c>
       <c r="I218" t="n">
-        <v>118</v>
+        <v>127.2333333333333</v>
       </c>
     </row>
     <row r="219">
@@ -8743,7 +9161,9 @@
       <c r="H219" t="n">
         <v>0.1215600924750089</v>
       </c>
-      <c r="I219" t="inlineStr"/>
+      <c r="I219" t="n">
+        <v>132.7916666666667</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -8774,7 +9194,9 @@
         <v>56.5</v>
       </c>
       <c r="H220" t="inlineStr"/>
-      <c r="I220" t="inlineStr"/>
+      <c r="I220" t="n">
+        <v>34.0820996870785</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -8807,7 +9229,9 @@
       <c r="H221" t="n">
         <v>0.501</v>
       </c>
-      <c r="I221" t="inlineStr"/>
+      <c r="I221" t="n">
+        <v>38.8183409385794</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -8840,7 +9264,9 @@
       <c r="H222" t="n">
         <v>0.498</v>
       </c>
-      <c r="I222" t="inlineStr"/>
+      <c r="I222" t="n">
+        <v>51.7928495263723</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -8873,7 +9299,9 @@
       <c r="H223" t="n">
         <v>0.465</v>
       </c>
-      <c r="I223" t="inlineStr"/>
+      <c r="I223" t="n">
+        <v>52.5071622623698</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -8906,7 +9334,9 @@
       <c r="H224" t="n">
         <v>0.441</v>
       </c>
-      <c r="I224" t="inlineStr"/>
+      <c r="I224" t="n">
+        <v>55.3644132056691</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -8939,7 +9369,9 @@
       <c r="H225" t="n">
         <v>0.467</v>
       </c>
-      <c r="I225" t="inlineStr"/>
+      <c r="I225" t="n">
+        <v>62.1163594444336</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -8972,7 +9404,9 @@
       <c r="H226" t="n">
         <v>0.44</v>
       </c>
-      <c r="I226" t="inlineStr"/>
+      <c r="I226" t="n">
+        <v>69.01064106942469</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -9005,7 +9439,9 @@
       <c r="H227" t="n">
         <v>0.447</v>
       </c>
-      <c r="I227" t="inlineStr"/>
+      <c r="I227" t="n">
+        <v>73.3196361410336</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -9038,7 +9474,9 @@
       <c r="H228" t="n">
         <v>0.407</v>
       </c>
-      <c r="I228" t="inlineStr"/>
+      <c r="I228" t="n">
+        <v>79.302189298518</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -9071,7 +9509,9 @@
       <c r="H229" t="n">
         <v>0.445</v>
       </c>
-      <c r="I229" t="inlineStr"/>
+      <c r="I229" t="n">
+        <v>83.14999999999999</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -9104,7 +9544,9 @@
       <c r="H230" t="n">
         <v>0.44</v>
       </c>
-      <c r="I230" t="inlineStr"/>
+      <c r="I230" t="n">
+        <v>85.24166666666666</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -9137,7 +9579,9 @@
       <c r="H231" t="n">
         <v>0.442</v>
       </c>
-      <c r="I231" t="inlineStr"/>
+      <c r="I231" t="n">
+        <v>92.80833333333334</v>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -9170,7 +9614,9 @@
       <c r="H232" t="n">
         <v>0.448</v>
       </c>
-      <c r="I232" t="inlineStr"/>
+      <c r="I232" t="n">
+        <v>98.425</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -9203,7 +9649,9 @@
       <c r="H233" t="n">
         <v>0.44</v>
       </c>
-      <c r="I233" t="inlineStr"/>
+      <c r="I233" t="n">
+        <v>104.9083333333334</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -9236,7 +9684,9 @@
       <c r="H234" t="n">
         <v>0.391</v>
       </c>
-      <c r="I234" t="inlineStr"/>
+      <c r="I234" t="n">
+        <v>110.4833333333333</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -9269,7 +9719,9 @@
       <c r="H235" t="n">
         <v>0.386</v>
       </c>
-      <c r="I235" t="inlineStr"/>
+      <c r="I235" t="n">
+        <v>115.15</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -9302,7 +9754,9 @@
       <c r="H236" t="n">
         <v>0.387</v>
       </c>
-      <c r="I236" t="inlineStr"/>
+      <c r="I236" t="n">
+        <v>121.4833333333333</v>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -9333,7 +9787,9 @@
         <v>12.9</v>
       </c>
       <c r="H237" t="inlineStr"/>
-      <c r="I237" t="inlineStr"/>
+      <c r="I237" t="n">
+        <v>120.1</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -9367,7 +9823,7 @@
         <v>0.382</v>
       </c>
       <c r="I238" t="n">
-        <v>120.7916666666667</v>
+        <v>127.2333333333333</v>
       </c>
     </row>
     <row r="239">
@@ -9401,7 +9857,9 @@
       <c r="H239" t="n">
         <v>0.143002971748049</v>
       </c>
-      <c r="I239" t="inlineStr"/>
+      <c r="I239" t="n">
+        <v>132.7916666666667</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -9430,7 +9888,9 @@
         <v>29.2</v>
       </c>
       <c r="H240" t="inlineStr"/>
-      <c r="I240" t="inlineStr"/>
+      <c r="I240" t="n">
+        <v>23.3563585414548</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -9461,7 +9921,9 @@
       <c r="H241" t="n">
         <v>0.507</v>
       </c>
-      <c r="I241" t="inlineStr"/>
+      <c r="I241" t="n">
+        <v>31.781255215535</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -9494,7 +9956,9 @@
       <c r="H242" t="n">
         <v>0.516</v>
       </c>
-      <c r="I242" t="inlineStr"/>
+      <c r="I242" t="n">
+        <v>34.0820996870785</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -9527,7 +9991,9 @@
       <c r="H243" t="n">
         <v>0.505</v>
       </c>
-      <c r="I243" t="inlineStr"/>
+      <c r="I243" t="n">
+        <v>38.8183409385794</v>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -9560,7 +10026,9 @@
       <c r="H244" t="n">
         <v>0.481</v>
       </c>
-      <c r="I244" t="inlineStr"/>
+      <c r="I244" t="n">
+        <v>51.7928495263723</v>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -9593,7 +10061,9 @@
       <c r="H245" t="n">
         <v>0.462</v>
       </c>
-      <c r="I245" t="inlineStr"/>
+      <c r="I245" t="n">
+        <v>52.5071622623698</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -9626,7 +10096,9 @@
       <c r="H246" t="n">
         <v>0.444</v>
       </c>
-      <c r="I246" t="inlineStr"/>
+      <c r="I246" t="n">
+        <v>55.3644132056691</v>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -9659,7 +10131,9 @@
       <c r="H247" t="n">
         <v>0.446</v>
       </c>
-      <c r="I247" t="inlineStr"/>
+      <c r="I247" t="n">
+        <v>62.1163594444336</v>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -9692,7 +10166,9 @@
       <c r="H248" t="n">
         <v>0.424</v>
       </c>
-      <c r="I248" t="inlineStr"/>
+      <c r="I248" t="n">
+        <v>69.01064106942469</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -9725,7 +10201,9 @@
       <c r="H249" t="n">
         <v>0.409</v>
       </c>
-      <c r="I249" t="inlineStr"/>
+      <c r="I249" t="n">
+        <v>73.3196361410336</v>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -9758,7 +10236,9 @@
       <c r="H250" t="n">
         <v>0.394</v>
       </c>
-      <c r="I250" t="inlineStr"/>
+      <c r="I250" t="n">
+        <v>79.302189298518</v>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -9791,7 +10271,9 @@
       <c r="H251" t="n">
         <v>0.423</v>
       </c>
-      <c r="I251" t="inlineStr"/>
+      <c r="I251" t="n">
+        <v>83.14999999999999</v>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -9824,7 +10306,9 @@
       <c r="H252" t="n">
         <v>0.443</v>
       </c>
-      <c r="I252" t="inlineStr"/>
+      <c r="I252" t="n">
+        <v>85.24166666666666</v>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -9857,7 +10341,9 @@
       <c r="H253" t="n">
         <v>0.418</v>
       </c>
-      <c r="I253" t="inlineStr"/>
+      <c r="I253" t="n">
+        <v>92.80833333333334</v>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -9890,7 +10376,9 @@
       <c r="H254" t="n">
         <v>0.424</v>
       </c>
-      <c r="I254" t="inlineStr"/>
+      <c r="I254" t="n">
+        <v>98.425</v>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -9923,7 +10411,9 @@
       <c r="H255" t="n">
         <v>0.396</v>
       </c>
-      <c r="I255" t="inlineStr"/>
+      <c r="I255" t="n">
+        <v>104.9083333333334</v>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -9956,7 +10446,9 @@
       <c r="H256" t="n">
         <v>0.379</v>
       </c>
-      <c r="I256" t="inlineStr"/>
+      <c r="I256" t="n">
+        <v>110.4833333333333</v>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -9989,7 +10481,9 @@
       <c r="H257" t="n">
         <v>0.372</v>
       </c>
-      <c r="I257" t="inlineStr"/>
+      <c r="I257" t="n">
+        <v>115.15</v>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -10022,7 +10516,9 @@
       <c r="H258" t="n">
         <v>0.393</v>
       </c>
-      <c r="I258" t="inlineStr"/>
+      <c r="I258" t="n">
+        <v>121.4833333333333</v>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -10053,7 +10549,9 @@
         <v>1.7</v>
       </c>
       <c r="H259" t="inlineStr"/>
-      <c r="I259" t="inlineStr"/>
+      <c r="I259" t="n">
+        <v>120.1</v>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -10087,7 +10585,7 @@
         <v>0.361</v>
       </c>
       <c r="I260" t="n">
-        <v>132.0833333333333</v>
+        <v>127.2333333333333</v>
       </c>
     </row>
     <row r="261">
@@ -10121,7 +10619,9 @@
       <c r="H261" t="n">
         <v>0.1283891254425096</v>
       </c>
-      <c r="I261" t="inlineStr"/>
+      <c r="I261" t="n">
+        <v>132.7916666666667</v>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -10150,7 +10650,9 @@
         <v>68.90000000000001</v>
       </c>
       <c r="H262" t="inlineStr"/>
-      <c r="I262" t="inlineStr"/>
+      <c r="I262" t="n">
+        <v>23.3563585414548</v>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -10181,7 +10683,9 @@
       <c r="H263" t="n">
         <v>0.502</v>
       </c>
-      <c r="I263" t="inlineStr"/>
+      <c r="I263" t="n">
+        <v>31.781255215535</v>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -10214,7 +10718,9 @@
       <c r="H264" t="n">
         <v>0.482</v>
       </c>
-      <c r="I264" t="inlineStr"/>
+      <c r="I264" t="n">
+        <v>34.0820996870785</v>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -10247,7 +10753,9 @@
       <c r="H265" t="n">
         <v>0.458</v>
       </c>
-      <c r="I265" t="inlineStr"/>
+      <c r="I265" t="n">
+        <v>38.8183409385794</v>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -10280,7 +10788,9 @@
       <c r="H266" t="n">
         <v>0.461</v>
       </c>
-      <c r="I266" t="inlineStr"/>
+      <c r="I266" t="n">
+        <v>51.7928495263723</v>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -10313,7 +10823,9 @@
       <c r="H267" t="n">
         <v>0.478</v>
       </c>
-      <c r="I267" t="inlineStr"/>
+      <c r="I267" t="n">
+        <v>52.5071622623698</v>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -10346,7 +10858,9 @@
       <c r="H268" t="n">
         <v>0.459</v>
       </c>
-      <c r="I268" t="inlineStr"/>
+      <c r="I268" t="n">
+        <v>55.3644132056691</v>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -10379,7 +10893,9 @@
       <c r="H269" t="n">
         <v>0.448</v>
       </c>
-      <c r="I269" t="inlineStr"/>
+      <c r="I269" t="n">
+        <v>62.1163594444336</v>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -10412,7 +10928,9 @@
       <c r="H270" t="n">
         <v>0.464</v>
       </c>
-      <c r="I270" t="inlineStr"/>
+      <c r="I270" t="n">
+        <v>69.01064106942469</v>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -10445,7 +10963,9 @@
       <c r="H271" t="n">
         <v>0.466</v>
       </c>
-      <c r="I271" t="inlineStr"/>
+      <c r="I271" t="n">
+        <v>73.3196361410336</v>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -10478,7 +10998,9 @@
       <c r="H272" t="n">
         <v>0.44</v>
       </c>
-      <c r="I272" t="inlineStr"/>
+      <c r="I272" t="n">
+        <v>79.302189298518</v>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -10511,7 +11033,9 @@
       <c r="H273" t="n">
         <v>0.424</v>
       </c>
-      <c r="I273" t="inlineStr"/>
+      <c r="I273" t="n">
+        <v>83.14999999999999</v>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -10544,7 +11068,9 @@
       <c r="H274" t="n">
         <v>0.443</v>
       </c>
-      <c r="I274" t="inlineStr"/>
+      <c r="I274" t="n">
+        <v>85.24166666666666</v>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -10577,7 +11103,9 @@
       <c r="H275" t="n">
         <v>0.399</v>
       </c>
-      <c r="I275" t="inlineStr"/>
+      <c r="I275" t="n">
+        <v>92.80833333333334</v>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -10610,7 +11138,9 @@
       <c r="H276" t="n">
         <v>0.418</v>
       </c>
-      <c r="I276" t="inlineStr"/>
+      <c r="I276" t="n">
+        <v>98.425</v>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -10643,7 +11173,9 @@
       <c r="H277" t="n">
         <v>0.426</v>
       </c>
-      <c r="I277" t="inlineStr"/>
+      <c r="I277" t="n">
+        <v>104.9083333333334</v>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -10676,7 +11208,9 @@
       <c r="H278" t="n">
         <v>0.36</v>
       </c>
-      <c r="I278" t="inlineStr"/>
+      <c r="I278" t="n">
+        <v>110.4833333333333</v>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -10709,7 +11243,9 @@
       <c r="H279" t="n">
         <v>0.328</v>
       </c>
-      <c r="I279" t="inlineStr"/>
+      <c r="I279" t="n">
+        <v>115.15</v>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -10742,7 +11278,9 @@
       <c r="H280" t="n">
         <v>0.335</v>
       </c>
-      <c r="I280" t="inlineStr"/>
+      <c r="I280" t="n">
+        <v>121.4833333333333</v>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -10773,7 +11311,9 @@
         <v>12</v>
       </c>
       <c r="H281" t="inlineStr"/>
-      <c r="I281" t="inlineStr"/>
+      <c r="I281" t="n">
+        <v>120.1</v>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -10807,7 +11347,7 @@
         <v>0.326</v>
       </c>
       <c r="I282" t="n">
-        <v>123.1666666666667</v>
+        <v>127.2333333333333</v>
       </c>
     </row>
     <row r="283">
@@ -10841,7 +11381,9 @@
       <c r="H283" t="n">
         <v>0.05754435877579889</v>
       </c>
-      <c r="I283" t="inlineStr"/>
+      <c r="I283" t="n">
+        <v>132.7916666666667</v>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -10870,7 +11412,9 @@
       </c>
       <c r="G284" t="inlineStr"/>
       <c r="H284" t="inlineStr"/>
-      <c r="I284" t="inlineStr"/>
+      <c r="I284" t="n">
+        <v>34.0820996870785</v>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -10903,7 +11447,9 @@
       <c r="H285" t="n">
         <v>0.486</v>
       </c>
-      <c r="I285" t="inlineStr"/>
+      <c r="I285" t="n">
+        <v>51.7928495263723</v>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -10936,7 +11482,9 @@
       <c r="H286" t="n">
         <v>0.465</v>
       </c>
-      <c r="I286" t="inlineStr"/>
+      <c r="I286" t="n">
+        <v>52.5071622623698</v>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -10969,7 +11517,9 @@
       <c r="H287" t="n">
         <v>0.428</v>
       </c>
-      <c r="I287" t="inlineStr"/>
+      <c r="I287" t="n">
+        <v>55.3644132056691</v>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -11002,7 +11552,9 @@
       <c r="H288" t="n">
         <v>0.443</v>
       </c>
-      <c r="I288" t="inlineStr"/>
+      <c r="I288" t="n">
+        <v>62.1163594444336</v>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -11035,7 +11587,9 @@
       <c r="H289" t="n">
         <v>0.423</v>
       </c>
-      <c r="I289" t="inlineStr"/>
+      <c r="I289" t="n">
+        <v>69.01064106942469</v>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -11068,7 +11622,9 @@
       <c r="H290" t="n">
         <v>0.417</v>
       </c>
-      <c r="I290" t="inlineStr"/>
+      <c r="I290" t="n">
+        <v>73.3196361410336</v>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -11101,7 +11657,9 @@
       <c r="H291" t="n">
         <v>0.414</v>
       </c>
-      <c r="I291" t="inlineStr"/>
+      <c r="I291" t="n">
+        <v>79.302189298518</v>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -11134,7 +11692,9 @@
       <c r="H292" t="n">
         <v>0.448</v>
       </c>
-      <c r="I292" t="inlineStr"/>
+      <c r="I292" t="n">
+        <v>83.14999999999999</v>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -11167,7 +11727,9 @@
       <c r="H293" t="n">
         <v>0.467</v>
       </c>
-      <c r="I293" t="inlineStr"/>
+      <c r="I293" t="n">
+        <v>85.24166666666666</v>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -11200,7 +11762,9 @@
       <c r="H294" t="n">
         <v>0.446</v>
       </c>
-      <c r="I294" t="inlineStr"/>
+      <c r="I294" t="n">
+        <v>92.80833333333334</v>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -11233,7 +11797,9 @@
       <c r="H295" t="n">
         <v>0.374</v>
       </c>
-      <c r="I295" t="inlineStr"/>
+      <c r="I295" t="n">
+        <v>98.425</v>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -11266,7 +11832,9 @@
       <c r="H296" t="n">
         <v>0.442</v>
       </c>
-      <c r="I296" t="inlineStr"/>
+      <c r="I296" t="n">
+        <v>104.9083333333334</v>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -11299,7 +11867,9 @@
       <c r="H297" t="n">
         <v>0.407</v>
       </c>
-      <c r="I297" t="inlineStr"/>
+      <c r="I297" t="n">
+        <v>110.4833333333333</v>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -11332,7 +11902,9 @@
       <c r="H298" t="n">
         <v>0.378</v>
       </c>
-      <c r="I298" t="inlineStr"/>
+      <c r="I298" t="n">
+        <v>115.15</v>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -11365,7 +11937,9 @@
       <c r="H299" t="n">
         <v>0.35</v>
       </c>
-      <c r="I299" t="inlineStr"/>
+      <c r="I299" t="n">
+        <v>121.4833333333333</v>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -11396,7 +11970,9 @@
         <v>0.4</v>
       </c>
       <c r="H300" t="inlineStr"/>
-      <c r="I300" t="inlineStr"/>
+      <c r="I300" t="n">
+        <v>120.1</v>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -11430,7 +12006,7 @@
         <v>0.38</v>
       </c>
       <c r="I301" t="n">
-        <v>128.475</v>
+        <v>127.2333333333333</v>
       </c>
     </row>
     <row r="302">
@@ -11464,7 +12040,9 @@
       <c r="H302" t="n">
         <v>0.1190151196048226</v>
       </c>
-      <c r="I302" t="inlineStr"/>
+      <c r="I302" t="n">
+        <v>132.7916666666667</v>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -11497,7 +12075,9 @@
       <c r="H303" t="n">
         <v>0.388</v>
       </c>
-      <c r="I303" t="inlineStr"/>
+      <c r="I303" t="n">
+        <v>92.80833333333334</v>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -11530,7 +12110,9 @@
       <c r="H304" t="n">
         <v>0.387</v>
       </c>
-      <c r="I304" t="inlineStr"/>
+      <c r="I304" t="n">
+        <v>98.425</v>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -11563,7 +12145,9 @@
       <c r="H305" t="n">
         <v>0.383</v>
       </c>
-      <c r="I305" t="inlineStr"/>
+      <c r="I305" t="n">
+        <v>104.9083333333334</v>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -11596,7 +12180,9 @@
       <c r="H306" t="n">
         <v>0.385</v>
       </c>
-      <c r="I306" t="inlineStr"/>
+      <c r="I306" t="n">
+        <v>110.4833333333333</v>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -11629,7 +12215,9 @@
       <c r="H307" t="n">
         <v>0.398</v>
       </c>
-      <c r="I307" t="inlineStr"/>
+      <c r="I307" t="n">
+        <v>115.15</v>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -11662,7 +12250,9 @@
       <c r="H308" t="n">
         <v>0.333</v>
       </c>
-      <c r="I308" t="inlineStr"/>
+      <c r="I308" t="n">
+        <v>121.4833333333333</v>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -11693,7 +12283,9 @@
         <v>5.2</v>
       </c>
       <c r="H309" t="inlineStr"/>
-      <c r="I309" t="inlineStr"/>
+      <c r="I309" t="n">
+        <v>120.1</v>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -11727,7 +12319,7 @@
         <v>0.3</v>
       </c>
       <c r="I310" t="n">
-        <v>120.5666666666667</v>
+        <v>127.2333333333333</v>
       </c>
     </row>
     <row r="311">
@@ -11761,7 +12353,9 @@
       <c r="H311" t="n">
         <v>0</v>
       </c>
-      <c r="I311" t="inlineStr"/>
+      <c r="I311" t="n">
+        <v>132.7916666666667</v>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -11794,7 +12388,9 @@
       <c r="H312" t="n">
         <v>0.362</v>
       </c>
-      <c r="I312" t="inlineStr"/>
+      <c r="I312" t="n">
+        <v>92.80833333333334</v>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -11827,7 +12423,9 @@
       <c r="H313" t="n">
         <v>0.342</v>
       </c>
-      <c r="I313" t="inlineStr"/>
+      <c r="I313" t="n">
+        <v>98.425</v>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -11860,7 +12458,9 @@
       <c r="H314" t="n">
         <v>0.305</v>
       </c>
-      <c r="I314" t="inlineStr"/>
+      <c r="I314" t="n">
+        <v>104.9083333333334</v>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -11893,7 +12493,9 @@
       <c r="H315" t="n">
         <v>0.374</v>
       </c>
-      <c r="I315" t="inlineStr"/>
+      <c r="I315" t="n">
+        <v>110.4833333333333</v>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -11926,7 +12528,9 @@
       <c r="H316" t="n">
         <v>0.369</v>
       </c>
-      <c r="I316" t="inlineStr"/>
+      <c r="I316" t="n">
+        <v>115.15</v>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -11959,7 +12563,9 @@
       <c r="H317" t="n">
         <v>0.361</v>
       </c>
-      <c r="I317" t="inlineStr"/>
+      <c r="I317" t="n">
+        <v>121.4833333333333</v>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -11990,7 +12596,9 @@
         <v>0.2</v>
       </c>
       <c r="H318" t="inlineStr"/>
-      <c r="I318" t="inlineStr"/>
+      <c r="I318" t="n">
+        <v>120.1</v>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -12024,7 +12632,7 @@
         <v>0.368</v>
       </c>
       <c r="I319" t="n">
-        <v>133.825</v>
+        <v>127.2333333333333</v>
       </c>
     </row>
     <row r="320">
@@ -12058,7 +12666,9 @@
       <c r="H320" t="n">
         <v>0</v>
       </c>
-      <c r="I320" t="inlineStr"/>
+      <c r="I320" t="n">
+        <v>132.7916666666667</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14259,785 +14869,547 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:B67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>state_code</t>
+          <t>year</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>state</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
           <t>cpi_overall</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>JHR</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Johor</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
+      <c r="A2" t="n">
+        <v>1960</v>
+      </c>
+      <c r="B2" t="n">
+        <v>21.3092412797334</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1961</v>
+      </c>
+      <c r="B3" t="n">
+        <v>21.2707977630436</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1962</v>
+      </c>
+      <c r="B4" t="n">
+        <v>21.2938638731113</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1963</v>
+      </c>
+      <c r="B5" t="n">
+        <v>21.9550923595525</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1964</v>
+      </c>
+      <c r="B6" t="n">
+        <v>21.8666722711776</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1965</v>
+      </c>
+      <c r="B7" t="n">
+        <v>21.8436061611484</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1966</v>
+      </c>
+      <c r="B8" t="n">
+        <v>22.0550455027883</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1967</v>
+      </c>
+      <c r="B9" t="n">
+        <v>23.0641878148471</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>1968</v>
+      </c>
+      <c r="B10" t="n">
+        <v>23.0276664740477</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>1969</v>
+      </c>
+      <c r="B11" t="n">
+        <v>22.9334798581942</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>1970</v>
+      </c>
+      <c r="B12" t="n">
+        <v>23.3563585414548</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>1971</v>
+      </c>
+      <c r="B13" t="n">
+        <v>23.7331050045995</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>1972</v>
+      </c>
+      <c r="B14" t="n">
+        <v>24.5000531617548</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>1973</v>
+      </c>
+      <c r="B15" t="n">
+        <v>27.0873018323506</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>1974</v>
+      </c>
+      <c r="B16" t="n">
+        <v>31.781255215535</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>1975</v>
+      </c>
+      <c r="B17" t="n">
+        <v>33.2075096832608</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>1976</v>
+      </c>
+      <c r="B18" t="n">
+        <v>34.0820996870785</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>1977</v>
+      </c>
+      <c r="B19" t="n">
+        <v>35.7140269689273</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>1978</v>
+      </c>
+      <c r="B20" t="n">
+        <v>37.4497517457152</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>1979</v>
+      </c>
+      <c r="B21" t="n">
+        <v>38.8183409385794</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>1980</v>
+      </c>
+      <c r="B22" t="n">
+        <v>41.4094339608595</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>1981</v>
+      </c>
+      <c r="B23" t="n">
+        <v>45.4261490550629</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>1982</v>
+      </c>
+      <c r="B24" t="n">
+        <v>48.0694512559551</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>1983</v>
+      </c>
+      <c r="B25" t="n">
+        <v>49.8500569163408</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>1984</v>
+      </c>
+      <c r="B26" t="n">
+        <v>51.7928495263723</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="B27" t="n">
+        <v>51.9722904068005</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>1986</v>
+      </c>
+      <c r="B28" t="n">
+        <v>52.3553276711112</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>1987</v>
+      </c>
+      <c r="B29" t="n">
+        <v>52.5071622623698</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>1988</v>
+      </c>
+      <c r="B30" t="n">
+        <v>53.8495180799345</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>1989</v>
+      </c>
+      <c r="B31" t="n">
+        <v>55.3644132056691</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>1990</v>
+      </c>
+      <c r="B32" t="n">
+        <v>56.8137433942992</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>1991</v>
+      </c>
+      <c r="B33" t="n">
+        <v>59.2898757105672</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>1992</v>
+      </c>
+      <c r="B34" t="n">
+        <v>62.1163594444336</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>1993</v>
+      </c>
+      <c r="B35" t="n">
+        <v>64.3131575223467</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>1994</v>
+      </c>
+      <c r="B36" t="n">
+        <v>66.7088037021399</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>1995</v>
+      </c>
+      <c r="B37" t="n">
+        <v>69.01064106942469</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>1996</v>
+      </c>
+      <c r="B38" t="n">
+        <v>71.4181183158851</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>1997</v>
+      </c>
+      <c r="B39" t="n">
+        <v>73.3196361410336</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>1998</v>
+      </c>
+      <c r="B40" t="n">
+        <v>77.18383172137879</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>1999</v>
+      </c>
+      <c r="B41" t="n">
+        <v>79.302189298518</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B42" t="n">
+        <v>80.55</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>2001</v>
+      </c>
+      <c r="B43" t="n">
+        <v>81.68333333333334</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>2002</v>
+      </c>
+      <c r="B44" t="n">
+        <v>83.14999999999999</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B45" t="n">
+        <v>84.05833333333334</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B46" t="n">
+        <v>85.24166666666666</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B47" t="n">
+        <v>87.77499999999999</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B48" t="n">
+        <v>90.95</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B49" t="n">
+        <v>92.80833333333334</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B50" t="n">
+        <v>97.84166666666664</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B51" t="n">
+        <v>98.425</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B52" t="n">
+        <v>100.0166666666667</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>2011</v>
+      </c>
+      <c r="B53" t="n">
+        <v>103.2</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>2012</v>
+      </c>
+      <c r="B54" t="n">
+        <v>104.9083333333334</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>2013</v>
+      </c>
+      <c r="B55" t="n">
+        <v>107.1166666666667</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B56" t="n">
+        <v>110.4833333333333</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B57" t="n">
+        <v>112.8083333333333</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>2016</v>
+      </c>
+      <c r="B58" t="n">
+        <v>115.15</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>2017</v>
+      </c>
+      <c r="B59" t="n">
+        <v>119.525</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B60" t="n">
+        <v>120.6833333333333</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B61" t="n">
+        <v>121.4833333333333</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B62" t="n">
+        <v>120.1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
         <v>2021</v>
       </c>
-      <c r="D2" t="n">
-        <v>126.3</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>JHR</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Johor</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
+      <c r="B63" t="n">
+        <v>123.075</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
         <v>2022</v>
       </c>
-      <c r="D3" t="n">
-        <v>130.625</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>JHR</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Johor</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
+      <c r="B64" t="n">
+        <v>127.2333333333333</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
         <v>2023</v>
       </c>
-      <c r="D4" t="n">
-        <v>133.5125</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>KDH</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Kedah</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>2021</v>
-      </c>
-      <c r="D5" t="n">
-        <v>120.3583333333333</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>KDH</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Kedah</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>2022</v>
-      </c>
-      <c r="D6" t="n">
-        <v>123.475</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>KDH</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Kedah</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D7" t="n">
-        <v>125.375</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>KTN</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Kelantan</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>2021</v>
-      </c>
-      <c r="D8" t="n">
-        <v>122.475</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>KTN</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Kelantan</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>2022</v>
-      </c>
-      <c r="D9" t="n">
-        <v>125.875</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>KTN</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Kelantan</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D10" t="n">
-        <v>127.875</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>MLK</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Melaka</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>2021</v>
-      </c>
-      <c r="D11" t="n">
-        <v>120.8583333333333</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>MLK</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Melaka</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>2022</v>
-      </c>
-      <c r="D12" t="n">
-        <v>124.1916666666667</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>MLK</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Melaka</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D13" t="n">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>PHG</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Pahang</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>2021</v>
-      </c>
-      <c r="D14" t="n">
-        <v>121.075</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>PHG</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Pahang</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>2022</v>
-      </c>
-      <c r="D15" t="n">
-        <v>124.6833333333333</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>PHG</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Pahang</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D16" t="n">
-        <v>127.8125</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>PRK</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Perak</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>2021</v>
-      </c>
-      <c r="D17" t="n">
-        <v>119.1</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>PRK</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Perak</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>2022</v>
-      </c>
-      <c r="D18" t="n">
-        <v>122.95</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>PRK</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Perak</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D19" t="n">
-        <v>126.1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>PLS</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Perlis</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>2021</v>
-      </c>
-      <c r="D20" t="n">
-        <v>116.4583333333333</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>PLS</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Perlis</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>2022</v>
-      </c>
-      <c r="D21" t="n">
-        <v>120.1666666666667</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>PLS</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Perlis</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D22" t="n">
-        <v>122.45</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>SBH</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Sabah</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>2021</v>
-      </c>
-      <c r="D23" t="n">
-        <v>114.6166666666667</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>SBH</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Sabah</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>2022</v>
-      </c>
-      <c r="D24" t="n">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>SBH</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Sabah</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D25" t="n">
-        <v>120.4875</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>SWK</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Sarawak</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>2021</v>
-      </c>
-      <c r="D26" t="n">
-        <v>117.475</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>SWK</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Sarawak</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>2022</v>
-      </c>
-      <c r="D27" t="n">
-        <v>120.7916666666667</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>SWK</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Sarawak</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D28" t="n">
-        <v>124.175</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>SGR</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Selangor</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>2021</v>
-      </c>
-      <c r="D29" t="n">
-        <v>126.7916666666667</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>SGR</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Selangor</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>2022</v>
-      </c>
-      <c r="D30" t="n">
-        <v>132.0833333333333</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>SGR</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Selangor</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D31" t="n">
-        <v>135.5375</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>TRG</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Terengganu</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>2021</v>
-      </c>
-      <c r="D32" t="n">
-        <v>119.525</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>TRG</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Terengganu</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>2022</v>
-      </c>
-      <c r="D33" t="n">
-        <v>123.1666666666667</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>TRG</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Terengganu</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D34" t="n">
-        <v>125.2125</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>KUL</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>W.P. Kuala Lumpur</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>2021</v>
-      </c>
-      <c r="D35" t="n">
-        <v>124.7333333333333</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>KUL</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>W.P. Kuala Lumpur</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>2022</v>
-      </c>
-      <c r="D36" t="n">
-        <v>128.475</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>KUL</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>W.P. Kuala Lumpur</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D37" t="n">
-        <v>130.9875</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>LBN</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>W.P. Labuan</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>2021</v>
-      </c>
-      <c r="D38" t="n">
-        <v>117.8333333333333</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>LBN</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>W.P. Labuan</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>2022</v>
-      </c>
-      <c r="D39" t="n">
-        <v>120.5666666666667</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>LBN</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>W.P. Labuan</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D40" t="n">
-        <v>122.25</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>PJY</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>W.P. Putrajaya</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>2021</v>
-      </c>
-      <c r="D41" t="n">
-        <v>124.7333333333333</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>PJY</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>W.P. Putrajaya</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>2022</v>
-      </c>
-      <c r="D42" t="n">
-        <v>133.825</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>PJY</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>W.P. Putrajaya</t>
-        </is>
-      </c>
-      <c r="C43" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D43" t="n">
-        <v>137.95</v>
+      <c r="B65" t="n">
+        <v>130.4</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B66" t="n">
+        <v>132.7916666666667</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B67" t="n">
+        <v>134.625</v>
       </c>
     </row>
   </sheetData>

</xml_diff>